<commit_message>
Add published project links
</commit_message>
<xml_diff>
--- a/Solar_PV_Sizing_Calculator.xlsx
+++ b/Solar_PV_Sizing_Calculator.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R46aafb3dfa674e8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Inputs" sheetId="2" r:id="R88d68545293047c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Consumo" sheetId="3" r:id="Rac0ad66530e64daf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Recurso_Solar" sheetId="4" r:id="R1b2718e8e2524be3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Modulo" sheetId="5" r:id="Rc81fe09d02c2457a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Inversor" sheetId="6" r:id="R8015b1edec664781"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Dimensionamento" sheetId="7" r:id="R2c524289c10a401e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Strings" sheetId="8" r:id="R23610aa491a6418b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Geracao" sheetId="9" r:id="Re20b792140de489a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Validacoes" sheetId="10" r:id="Ree2ddd709e3d452b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Premissas" sheetId="11" r:id="Rdc6530dadb4c438f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Documentacao" sheetId="12" r:id="R31445446f9b84667"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R603980bd34bc48af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Inputs" sheetId="2" r:id="R91497ceb3d804d35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Consumo" sheetId="3" r:id="R7e6c6075752d4a82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Recurso_Solar" sheetId="4" r:id="R2d900ebaa27d4765"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Modulo" sheetId="5" r:id="R761442697d224e27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Inversor" sheetId="6" r:id="R79f6e9a31ae2461e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Dimensionamento" sheetId="7" r:id="Rbdb77cf245ef4072"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Strings" sheetId="8" r:id="Ra98b85221b27496f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Geracao" sheetId="9" r:id="Rfe6e9032650549e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Validacoes" sheetId="10" r:id="Raf3bf19903974e05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Premissas" sheetId="11" r:id="R695f3f795ecc419b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Documentacao" sheetId="12" r:id="R9b066f11b65a4c4f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1398,7 +1398,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbaa0cb4df1d74946"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd2a856e0d2584ae5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1428,7 +1428,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R484ac5fb81d14dca"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbac9c4b492ef4e4a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1463,7 +1463,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbc5abd3ffaf04fab"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3f86513b42f04c2c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1498,7 +1498,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2239d2c421964627"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R04c243d91560498e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1528,7 +1528,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9436a8ec4af94b0a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra9153bc6e8c644ce"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -5176,7 +5176,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf08efb055aa14d12"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8614456c0644990"/>
 </x:worksheet>
 </file>
 
@@ -26052,7 +26052,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c301790047b4df8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27576129648c43e4"/>
 </x:worksheet>
 </file>
 
@@ -43638,6 +43638,6 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26c93e59119544f0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75aab27a17014d6b"/>
 </x:worksheet>
 </file>
</xml_diff>